<commit_message>
auto sync 2026-10-07 18:38 KST
</commit_message>
<xml_diff>
--- a/봉제현황/생산평균_애리후세_20261007.xlsx
+++ b/봉제현황/생산평균_애리후세_20261007.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>534</v>
+        <v>527.6</v>
       </c>
     </row>
     <row r="4">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24030</v>
+        <v>24270</v>
       </c>
     </row>
     <row r="6">
@@ -481,7 +481,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-18–2026-10-06</t>
+          <t>2026-06-18–2026-10-07</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>파일명우선(본문날짜칸공란):9/21·9/22·9/28; 일요일·공휴일(추석9/24–9/26·10/5)KPI제외; 9/28=540(460+80 총합계); 9/29=582; 9/30=683; 10/1=607; 10/2=404; 10/3=323(지정근무일); 10/6=240; 10/7=판독보류(240/230, null·KPI제외)</t>
+          <t>파일명우선(본문날짜칸공란):9/21·9/22·9/28; 일요일·공휴일(추석9/24–9/26·10/5)KPI제외; 9/28=540(460+80 총합계); 9/29=582; 9/30=683; 10/1=607; 10/2=404; 10/3=323(지정근무일); 10/6=240; 10/7=240(사용자 확정 2026-10-07 18:30)</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1200,6 +1200,21 @@
       <c r="C46" t="inlineStr">
         <is>
           <t>10/6·화</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>240</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10/7·수</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1526,7 +1541,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>393.5</v>
+        <v>362.8</v>
       </c>
     </row>
     <row r="3">
@@ -1536,7 +1551,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1547,7 +1562,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-01–2026-10-06</t>
+          <t>2026-10-01–2026-10-07</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1581,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10/6</t>
+          <t>10/7</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1576,30 +1591,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10/3</t>
+          <t>10/6</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>323</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10/2</t>
+          <t>10/3</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>404</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>10/2</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>10/1</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B10" t="n">
         <v>607</v>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-07 18:45 KST
</commit_message>
<xml_diff>
--- a/봉제현황/생산평균_애리후세_20261007.xlsx
+++ b/봉제현황/생산평균_애리후세_20261007.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>527.6</v>
+        <v>528.5</v>
       </c>
     </row>
     <row r="4">
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24270</v>
+        <v>24310</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>파일명우선(본문날짜칸공란):9/21·9/22·9/28; 일요일·공휴일(추석9/24–9/26·10/5)KPI제외; 9/28=540(460+80 총합계); 9/29=582; 9/30=683; 10/1=607; 10/2=404; 10/3=323(지정근무일); 10/6=240; 10/7=240(사용자 확정 2026-10-07 18:30)</t>
+          <t>파일명우선(본문날짜칸공란):9/21·9/22·9/28; 일요일·공휴일(추석9/24–9/26·10/5)KPI제외; 9/28=540(460+80 총합계); 9/29=582; 9/30=683; 10/1=607; 10/2=404; 10/3=323(지정근무일); 10/6=240; 10/7=280(사용자 확정 2026-10-07 18:38 280 (18:30 240 정정))</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>362.8</v>
+        <v>370.8</v>
       </c>
     </row>
     <row r="3">
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7">

</xml_diff>